<commit_message>
U1 BPs: full address, contact, credit limit, BP group and price list details
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/u1_masters/U1_Master_Data.xlsx
+++ b/data/u1_masters/U1_Master_Data.xlsx
@@ -3651,17 +3651,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="33" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="42" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3677,32 +3687,82 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Billing / pay-to address</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Shipping address</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>State</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>City</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>PAN</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>GSTIN</t>
+          <t>GSTIN (dummy)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Payment terms (days)</t>
+          <t>PAN (dummy)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Buys</t>
+          <t>Payment terms</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Credit limit (INR)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Contact person</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>BP group</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Control account</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Price list</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>TDS code</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Buys / supplies</t>
         </is>
       </c>
     </row>
@@ -3719,28 +3779,78 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>No. 45, 2nd Floor, Prestige Arcade, Bannerghatta Road, JP Nagar, Bengaluru - 560076</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Site - Dabaspet Industrial Shed: Plot 12, KIADB Industrial Area, Dabaspet, Dabaspet - 562111</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>Karnataka</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>29AAHCH5521K1ZB</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>AAHCH5521K</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>29AAHCH5521K1ZB</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>45</v>
-      </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>Net 45 Days</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Suresh Kumar</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Purchase Manager</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>+91 90000 10001</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>accounts@hampiinfra.example</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>EPC &amp; Infra</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>5002-02-04-01</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Sales Price (Dummy - Restricted)</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
         <is>
           <t>Industrial sheds - roof trusses, columns</t>
         </is>
@@ -3759,28 +3869,78 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Kaveri House, 3rd Floor, Hunsur Road, Hebbal Industrial Area, Mysuru - 570016</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Site - Kaveri Park Phase 2: Survey No. 88, Nanjangud Industrial Area, Nanjangud, Nanjangud - 571301</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>Karnataka</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Mysuru</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>29AABCK7734M1ZZ</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>AABCK7734M</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>29AABCK7734M1ZZ</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>30</v>
-      </c>
       <c r="H3" t="inlineStr">
+        <is>
+          <t>Net 30 Days</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Lakshmi Narayan</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Projects Head</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>+91 90000 10002</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>accounts@kaveriparks.example</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Industrial Developer</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>5002-02-04-01</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Sales Price (Dummy - Restricted)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
         <is>
           <t>Factory buildings - structural steel</t>
         </is>
@@ -3799,28 +3959,78 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>8-2-293, Godavari Towers, Road No. 14, Banjara Hills, Hyderabad - 500034</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Site - 2x150 MW Power Plant: Sy. No. 210, Pashamylaram Industrial Area, Patancheru, Sangareddy - 502307</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>Telangana</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Hyderabad</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>36AAGCG4410P1ZE</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>AAGCG4410P</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>36AAGCG4410P1ZE</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>60</v>
-      </c>
       <c r="H4" t="inlineStr">
+        <is>
+          <t>Net 60 Days</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>7500000</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Venkat Reddy</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Procurement Manager</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>+91 90000 10003</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>accounts@godavaripower.example</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Power &amp; Process</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>5002-02-04-01</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Sales Price (Dummy - Restricted)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
         <is>
           <t>Pipe racks, platforms, base plates</t>
         </is>
@@ -3839,28 +4049,78 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>No. 18, Palar Plaza, Anna Salai, Teynampet, Chennai - 600018</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Site - Palar Logistics Park: Plot B-7, SIPCOT Industrial Park, Oragadam, Kancheepuram - 602105</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>Tamil Nadu</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Chennai</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>33AAPFP2287D1Z6</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>AAPFP2287D</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>33AAPFP2287D1Z6</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>45</v>
-      </c>
       <c r="H5" t="inlineStr">
+        <is>
+          <t>Net 45 Days</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>4000000</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Karthik Subramanian</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Purchase Manager</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>+91 90000 10004</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>accounts@palarlogistics.example</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Industrial Developer</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>5002-02-04-01</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Sales Price (Dummy - Restricted)</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
         <is>
           <t>PEB warehouses - trusses &amp; columns</t>
         </is>
@@ -3879,28 +4139,78 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Deccan House, 5th Floor, Senapati Bapat Road, Shivajinagar, Pune - 411016</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Site - Bhima River Bridge: NH-65, Km 42, Bhigwan Road, Indapur, Indapur - 413106</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>Maharashtra</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Pune</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>27AADCD9063R1ZW</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>AADCD9063R</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>27AADCD9063R1ZW</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>60</v>
-      </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>Net 60 Days</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Amit Deshpande</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>+91 90000 10005</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>accounts@deccanbridges.example</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>EPC &amp; Infra</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>5002-02-04-01</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Sales Price (Dummy - Restricted)</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
         <is>
           <t>Bridge girders, TMT &amp; site electricals</t>
         </is>
@@ -3917,18 +4227,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="39" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="43" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="43" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3944,37 +4263,82 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Billing / pay-to address</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Shipping address</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>State</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>City</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>PAN</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>GSTIN</t>
+          <t>GSTIN (dummy)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Payment terms (days)</t>
+          <t>PAN (dummy)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Payment terms</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Credit limit (INR)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Contact person</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Mobile</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>BP group</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Control account</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Price list</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>TDS code</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Supplies</t>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Buys / supplies</t>
         </is>
       </c>
     </row>
@@ -3991,33 +4355,78 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Plot 7, Tungabhadra Steel Yard, Hospet Road, Kurugodu Cross, Ballari - 583101</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Stock Yard: Plot 22, KIADB Industrial Area, Sanklapur, Hosapete - 583201</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>Karnataka</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Ballari</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>29AAKFT3318L1ZP</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
         <is>
           <t>AAKFT3318L</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>29AAKFT3318L1ZP</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>30</v>
-      </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>Net 30 Days</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Mahesh Gowda</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>+91 90000 10101</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>accounts@tungabhadrasteel.example</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Steel Suppliers</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>TMT bars, structural steel (194Q pending)</t>
         </is>
@@ -4036,33 +4445,78 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>No. 112, Chamundi Complex, Bannur Road, Alanahalli, Mysuru - 570028</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Crusher Unit: Sy. No. 45, Belagola Road, Srirangapatna Taluk, Srirangapatna - 571438</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>Karnataka</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Mysuru</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>29AAJFC6620B1ZP</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
         <is>
           <t>AAJFC6620B</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>29AAJFC6620B1ZP</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>15</v>
-      </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>Net 15 Days</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Ravi Shankar</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>+91 90000 10102</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>accounts@chamundicement.example</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Building Materials</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Cement, river sand, M-sand, aggregate</t>
         </is>
@@ -4081,33 +4535,78 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>No. 23, 1st Floor, Sadar Patrappa Road, Chickpet, Bengaluru - 560002</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Godown: No. 9, 4th Cross, Peenya 2nd Stage, Peenya, Bengaluru - 560058</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
           <t>Karnataka</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>29AAQFV1145H1ZT</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>AAQFV1145H</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>29AAQFV1145H1ZT</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>30</v>
-      </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>Net 30 Days</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Anil Rao</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Sales Executive</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>+91 90000 10103</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>accounts@vidyutelectricals.example</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>Elec &amp; Plumbing</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Cables, distribution boards, flood lights</t>
         </is>
@@ -4126,33 +4625,78 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>No. 56, Jalavahini Buildings, Avinashi Road, Peelamedu, Coimbatore - 641004</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Factory: SF No. 312, Kurichi Industrial Estate, Kurichi, Coimbatore - 641021</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
           <t>Tamil Nadu</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Coimbatore</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>33AAEFJ8872N1ZR</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>AAEFJ8872N</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>33AAEFJ8872N1ZR</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>30</v>
-      </c>
       <c r="H5" t="inlineStr">
         <is>
+          <t>Net 30 Days</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>800000</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Senthil Kumar</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>+91 90000 10104</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>accounts@jalavahinipipes.example</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Elec &amp; Plumbing</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>PVC and GI pipes</t>
         </is>
@@ -4171,33 +4715,78 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Unit 14, Rakshak Industrial Estate, LBS Marg, Ghatkopar West, Mumbai - 400086</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Warehouse: Gala 3, Bhiwandi Logistics Park, Mumbai-Nashik Highway, Bhiwandi, Bhiwandi - 421302</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
           <t>Maharashtra</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Mumbai</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>27AAMFR4409G1Z2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
         <is>
           <t>AAMFR4409G</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>27AAMFR4409G1Z2</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>30</v>
-      </c>
       <c r="H6" t="inlineStr">
         <is>
+          <t>Net 30 Days</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Priya Patil</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Key Account Manager</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>+91 90000 10105</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>accounts@rakshaksafety.example</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>Safety &amp; Consumable</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>Helmets, safety shoes, harness</t>
         </is>
@@ -4216,33 +4805,78 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>No. 77, 1st Main, Yeshwanthpur Industrial Suburb, Yeshwanthpur, Bengaluru - 560022</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Store: Plot 41, KIADB Industrial Area, Bommasandra, Bengaluru - 560099</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
           <t>Karnataka</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>29AABFA5536E1ZO</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>AABFA5536E</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>29AABFA5536E1ZO</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>15</v>
-      </c>
       <c r="H7" t="inlineStr">
         <is>
+          <t>Net 15 Days</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Manjunath H</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Sales Executive</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>+91 90000 10106</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>accounts@agniwelding.example</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>Safety &amp; Consumable</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>Welding rods, cutting &amp; grinding discs</t>
         </is>
@@ -4261,33 +4895,78 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>No. 5, Shakti Arcade, Station Road, Old Hubballi, Hubballi - 580020</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Warehouse: Plot 18, Gokul Road Industrial Area, Gokul Road, Hubballi - 580030</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
           <t>Karnataka</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Hubballi</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>29AAKFS2291C1Z3</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
         <is>
           <t>AAKFS2291C</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>29AAKFS2291C1Z3</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>30</v>
-      </c>
       <c r="H8" t="inlineStr">
         <is>
+          <t>Net 30 Days</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>700000</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Basavaraj Patil</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>+91 90000 10107</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>accounts@shaktitools.example</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Tools &amp; Equipment</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>Pumps, power tools, drills, epoxy grout</t>
         </is>
@@ -4306,33 +4985,78 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
+          <t>No. 3, Transport Nagar, Tumkur Road, Yeshwanthpur, Bengaluru - 560022</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Truck Terminal: Plot 61, Peenya 1st Stage, Peenya, Bengaluru - 560058</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
           <t>Karnataka</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Bengaluru</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>29AAGFS7740Q1ZA</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
         <is>
           <t>AAGFS7740Q</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>29AAGFS7740Q1ZA</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>15</v>
-      </c>
       <c r="H9" t="inlineStr">
         <is>
+          <t>Net 15 Days</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>300000</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Imran Khan</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Operations Manager</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>+91 90000 10108</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>accounts@sarathiroadlines.example</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Transporters</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
           <t>C2</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>Transport (GTA) - TDS 194C 2%</t>
         </is>
@@ -4351,33 +5075,78 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>Shed No. 11, Apparel Park Road, KIADB Industrial Area, Doddaballapur - 561203</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Workshop: Shed No. 12, Apparel Park Road, KIADB Industrial Area, Doddaballapur - 561203</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
           <t>Karnataka</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Doddaballapur</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>29BQRPR6153A1ZH</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
         <is>
           <t>BQRPR6153A</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>29BQRPR6153A1ZH</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>30</v>
-      </c>
       <c r="H10" t="inlineStr">
         <is>
+          <t>Net 30 Days</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Ramesh R</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Proprietor</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>+91 90000 10109</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>accounts@rameshfabrication.example</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Subcontractors</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
           <t>C1</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>Fabrication subcontracting - TDS 194C 1%</t>
         </is>

</xml_diff>

<commit_message>
Complete details on the 15 demo BPs (address, contact, credit limit, group, price list)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/u1_masters/U1_Master_Data.xlsx
+++ b/data/u1_masters/U1_Master_Data.xlsx
@@ -3651,7 +3651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:R12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3666,7 +3666,7 @@
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="21" customWidth="1" min="11" max="11"/>
     <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="33" customWidth="1" min="13" max="13"/>
+    <col width="39" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="17" customWidth="1" min="15" max="15"/>
     <col width="34" customWidth="1" min="16" max="16"/>
@@ -4213,6 +4213,516 @@
       <c r="R6" t="inlineStr">
         <is>
           <t>Bridge girders, TMT &amp; site electricals</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>C0001</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Sahyadri Infra Projects Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Sahyadri House, 7th Floor, Bandra Kurla Complex, Bandra East, Mumbai - 400051</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Site - Navi Mumbai Logistics Hub: Plot 18, TTC Industrial Area, Mahape, Navi Mumbai - 400710</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>27AAGCS6631P1ZQ</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>AAGCS6631P</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Net 45 Days</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>7500000</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Rahul Shinde</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Procurement Manager</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>+91 90000 20001</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>accounts@sahyadriinfra.example</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>EPC &amp; Infra</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>5002-02-04-01</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Sales Price (Dummy - Restricted)</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>C0002</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Coromandel Power Engineering Ltd</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Coromandel Towers, 4th Floor, Mount Road, Nandanam, Chennai - 600035</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Site - Ennore Power Station: Ennore Port Road, Ennore, Ennore, Chennai - 600057</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>33AABCC8842H1ZQ</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>AABCC8842H</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Net 60 Days</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>10000000</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Ganesan R</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Purchase Manager</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>+91 90000 20002</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>accounts@coromandelpower.example</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>Power &amp; Process</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>5002-02-04-01</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Sales Price (Dummy - Restricted)</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>C0003</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Vijayanagar Petrochem Industries Ltd</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Vijayanagar Petrochem Complex, Sandur Road, Toranagallu, Ballari - 583123</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Site - Refinery Expansion: Plant Gate 3, Sandur Road, Toranagallu, Ballari - 583123</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Karnataka</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>29AACCV2207N1Z3</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>AACCV2207N</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Net 45 Days</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Prasanna Hegde</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Materials Manager</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>+91 90000 20003</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>accounts@vijayanagarpetrochem.example</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Power &amp; Process</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>5002-02-04-01</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Sales Price (Dummy - Restricted)</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>C0004</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Nila Cement Works Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Nila Cement Works, Kanjikode Industrial Area, Kanjikode, Palakkad - 678621</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Site - Kiln Upgrade: Plant Gate 1, Kanjikode Industrial Area, Kanjikode, Palakkad - 678621</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Kerala</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>32AAICN4419D1ZT</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>AAICN4419D</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Net 30 Days</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Anoop Menon</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Purchase Manager</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>+91 90000 20004</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>accounts@nilacement.example</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Power &amp; Process</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>5002-02-04-01</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Sales Price (Dummy - Restricted)</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>C0005</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Telangana Urban Metro Contractors</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Plot 45, Metro Bhavan, Begumpet Road, Begumpet, Hyderabad - 500016</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Site - Metro Phase 2 Depot: Sy. No. 301, Miyapur Depot Road, Miyapur, Hyderabad - 500049</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>36AAFFT7753G1ZV</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>AAFFT7753G</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Net 60 Days</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>8000000</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Ramana Murthy</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>+91 90000 20005</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>accounts@telanganametro.example</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>EPC &amp; Infra</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>5002-02-04-01</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Sales Price (Dummy - Restricted)</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>C0006</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Hosur Auto Components Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Plot 88, SIPCOT Phase I, Bagalur Road, SIPCOT Industrial Area, Hosur - 635126</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Plant 2: Plot 92, SIPCOT Phase II, Mookandapalli, Hosur - 635126</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>33AAHCH3398F1ZI</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>AAHCH3398F</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Net 30 Days</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Vignesh K</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Purchase Manager</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>+91 90000 20006</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>accounts@hosurauto.example</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Manufacturing</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>5002-02-04-01</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Sales Price (Dummy - Restricted)</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
     </row>
@@ -4227,11 +4737,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:R19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="39" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
@@ -5152,6 +5662,771 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>V0001</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Shree Ganesh Steel Traders</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>No. 14, Shree Ganesh Complex, Old Madras Road, KR Puram, Bengaluru - 560036</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Stock Yard: Plot 5, Hoskote Industrial Area, Hoskote, Hoskote - 562114</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Karnataka</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>29AAKFS4821K1ZQ</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>AAKFS4821K</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Net 30 Days</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Ganesh Rao</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>+91 90000 20101</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>accounts@shreeganeshsteel.example</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Steel Suppliers</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Q01</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>V0002</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Deccan Structural Steels Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Plot 31, Deccan Steel House, IDA Jeedimetla, Jeedimetla, Hyderabad - 500055</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Rolling Yard: Sy. No. 120, Medchal Industrial Area, Medchal, Medchal - 501401</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>36AADCD7315M1ZG</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>AADCD7315M</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Net 45 Days</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>5000000</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Srinivas Rao</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>+91 90000 20102</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>accounts@deccanstructural.example</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Steel Suppliers</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Q01</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>V0003</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Kaveri Special Alloys LLP</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>No. 9, Kaveri Alloys Building, GST Road, Guindy Industrial Estate, Chennai - 600032</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Warehouse: Plot C-14, Ambattur Industrial Estate, Ambattur, Chennai - 600058</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>33AAQFK2290B1ZJ</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>AAQFK2290B</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Net 30 Days</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Arun Prakash</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Sales Head</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>+91 90000 20103</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>accounts@kaverialloys.example</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Steel Suppliers</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>V0004</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Nandi Welding Consumables</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>No. 41, 3rd Cross, Magadi Road, Kamakshipalya, Bengaluru - 560079</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Godown: No. 18, Peenya 3rd Phase, Peenya, Bengaluru - 560058</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Karnataka</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>29ABNPN6612R1ZQ</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>ABNPN6612R</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Net 15 Days</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Nagaraj N</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Proprietor</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>+91 90000 20104</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>accounts@nandiwelding.example</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Safety &amp; Consumable</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>V0005</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Vayu Industrial Gases</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Plot 22, Vayu Gas Plant, NH-48, Antharasanahalli Industrial Area, Tumakuru - 572106</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Cylinder Filling Station: Plot 23, NH-48, Antharasanahalli Industrial Area, Tumakuru - 572106</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Karnataka</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>29AAHCV3304L1Z2</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>AAHCV3304L</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Net 15 Days</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Kiran Kumar</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Plant Manager</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>+91 90000 20105</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>accounts@vayugases.example</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Safety &amp; Consumable</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>V0006</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Suraksha Safety Solutions</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Office 204, Suraksha Plaza, Mumbai-Pune Highway, Pimpri, Pune - 411018</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Warehouse: Gat No. 112, Chakan MIDC, Chakan, Pune - 410501</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>27AAPFS9087C1ZM</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>AAPFS9087C</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Net 30 Days</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Sneha Joshi</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Sales Manager</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>+91 90000 20106</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>accounts@surakshasafety.example</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Safety &amp; Consumable</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>V0007</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Bharathi Blasting &amp; Coating Works</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Shed No. 4, Bharathi Works, Tumkur Road, Nelamangala Industrial Area, Nelamangala - 562123</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Blasting Yard: Sy. No. 77, Tumkur Road, Nelamangala Industrial Area, Nelamangala - 562123</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Karnataka</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>29ACBPB4410J1Z0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>ACBPB4410J</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Net 30 Days</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>500000</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Bharath B</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Proprietor</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>+91 90000 20107</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>accounts@bharathicoating.example</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Subcontractors</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>V0008</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Mysore Freight Carriers</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>No. 8, Transport Layout, Hunsur Road, Hebbal, Mysuru - 570017</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Truck Terminal: Plot 9, Bengaluru-Mysuru Road, Bannimantap, Mysuru - 570015</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Karnataka</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>29AAJFM1176E1Z8</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>AAJFM1176E</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Net 15 Days</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>300000</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Mohammed Rafi</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Operations Manager</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>+91 90000 20108</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>accounts@mysorefreight.example</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Transporters</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>V0009</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Prakash &amp; Associates Chartered Engineers</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>No. 112, 2nd Floor, Prakash Chambers, Residency Road, Shanthala Nagar, Bengaluru - 560025</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Office: No. 112, 2nd Floor, Residency Road, Shanthala Nagar, Bengaluru - 560025</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Karnataka</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>29AAEFP5521Q1ZO</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>AAEFP5521Q</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Net 30 Days</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>200000</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Prakash S</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>+91 90000 20109</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>accounts@prakashassociates.example</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Consultants</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>3002-02-01</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Purchase Price (Dummy)</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>J10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove credit limits from all BPs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/u1_masters/U1_Master_Data.xlsx
+++ b/data/u1_masters/U1_Master_Data.xlsx
@@ -3651,7 +3651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R12"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3662,16 +3662,15 @@
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
     <col width="21" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="39" customWidth="1" min="13" max="13"/>
-    <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="17" customWidth="1" min="15" max="15"/>
-    <col width="34" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="42" customWidth="1" min="18" max="18"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="39" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="34" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="42" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3717,50 +3716,45 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Credit limit (INR)</t>
+          <t>Contact person</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Contact person</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>BP group</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>BP group</t>
+          <t>Control account</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Control account</t>
+          <t>Price list</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Price list</t>
+          <t>TDS code</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>TDS code</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Buys / supplies</t>
         </is>
@@ -3807,50 +3801,47 @@
           <t>Net 45 Days</t>
         </is>
       </c>
-      <c r="I2" t="n">
-        <v>5000000</v>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Suresh Kumar</t>
+        </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Suresh Kumar</t>
+          <t>Purchase Manager</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Purchase Manager</t>
+          <t>+91 90000 10001</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>+91 90000 10001</t>
+          <t>accounts@hampiinfra.example</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>accounts@hampiinfra.example</t>
+          <t>EPC &amp; Infra</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>EPC &amp; Infra</t>
+          <t>5002-02-04-01</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>5002-02-04-01</t>
+          <t>Sales Price (Dummy - Restricted)</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Sales Price (Dummy - Restricted)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
         <is>
           <t>Industrial sheds - roof trusses, columns</t>
         </is>
@@ -3897,50 +3888,47 @@
           <t>Net 30 Days</t>
         </is>
       </c>
-      <c r="I3" t="n">
-        <v>3000000</v>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Lakshmi Narayan</t>
+        </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Lakshmi Narayan</t>
+          <t>Projects Head</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Projects Head</t>
+          <t>+91 90000 10002</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>+91 90000 10002</t>
+          <t>accounts@kaveriparks.example</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>accounts@kaveriparks.example</t>
+          <t>Industrial Developer</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Industrial Developer</t>
+          <t>5002-02-04-01</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>5002-02-04-01</t>
+          <t>Sales Price (Dummy - Restricted)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Sales Price (Dummy - Restricted)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
         <is>
           <t>Factory buildings - structural steel</t>
         </is>
@@ -3987,50 +3975,47 @@
           <t>Net 60 Days</t>
         </is>
       </c>
-      <c r="I4" t="n">
-        <v>7500000</v>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Venkat Reddy</t>
+        </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Venkat Reddy</t>
+          <t>Procurement Manager</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
+          <t>+91 90000 10003</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>+91 90000 10003</t>
+          <t>accounts@godavaripower.example</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>accounts@godavaripower.example</t>
+          <t>Power &amp; Process</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Power &amp; Process</t>
+          <t>5002-02-04-01</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>5002-02-04-01</t>
+          <t>Sales Price (Dummy - Restricted)</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Sales Price (Dummy - Restricted)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
         <is>
           <t>Pipe racks, platforms, base plates</t>
         </is>
@@ -4077,50 +4062,47 @@
           <t>Net 45 Days</t>
         </is>
       </c>
-      <c r="I5" t="n">
-        <v>4000000</v>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Karthik Subramanian</t>
+        </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Karthik Subramanian</t>
+          <t>Purchase Manager</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Purchase Manager</t>
+          <t>+91 90000 10004</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>+91 90000 10004</t>
+          <t>accounts@palarlogistics.example</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>accounts@palarlogistics.example</t>
+          <t>Industrial Developer</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Industrial Developer</t>
+          <t>5002-02-04-01</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>5002-02-04-01</t>
+          <t>Sales Price (Dummy - Restricted)</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Sales Price (Dummy - Restricted)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
         <is>
           <t>PEB warehouses - trusses &amp; columns</t>
         </is>
@@ -4167,50 +4149,47 @@
           <t>Net 60 Days</t>
         </is>
       </c>
-      <c r="I6" t="n">
-        <v>10000000</v>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Amit Deshpande</t>
+        </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Amit Deshpande</t>
+          <t>Project Manager</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Project Manager</t>
+          <t>+91 90000 10005</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>+91 90000 10005</t>
+          <t>accounts@deccanbridges.example</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>accounts@deccanbridges.example</t>
+          <t>EPC &amp; Infra</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>EPC &amp; Infra</t>
+          <t>5002-02-04-01</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>5002-02-04-01</t>
+          <t>Sales Price (Dummy - Restricted)</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Sales Price (Dummy - Restricted)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
         <is>
           <t>Bridge girders, TMT &amp; site electricals</t>
         </is>
@@ -4257,45 +4236,42 @@
           <t>Net 45 Days</t>
         </is>
       </c>
-      <c r="I7" t="n">
-        <v>7500000</v>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Rahul Shinde</t>
+        </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Rahul Shinde</t>
+          <t>Procurement Manager</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
+          <t>+91 90000 20001</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>+91 90000 20001</t>
+          <t>accounts@sahyadriinfra.example</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>accounts@sahyadriinfra.example</t>
+          <t>EPC &amp; Infra</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>EPC &amp; Infra</t>
+          <t>5002-02-04-01</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>5002-02-04-01</t>
+          <t>Sales Price (Dummy - Restricted)</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
-        <is>
-          <t>Sales Price (Dummy - Restricted)</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4342,45 +4318,42 @@
           <t>Net 60 Days</t>
         </is>
       </c>
-      <c r="I8" t="n">
-        <v>10000000</v>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Ganesan R</t>
+        </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Ganesan R</t>
+          <t>Purchase Manager</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Purchase Manager</t>
+          <t>+91 90000 20002</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>+91 90000 20002</t>
+          <t>accounts@coromandelpower.example</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>accounts@coromandelpower.example</t>
+          <t>Power &amp; Process</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Power &amp; Process</t>
+          <t>5002-02-04-01</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>5002-02-04-01</t>
+          <t>Sales Price (Dummy - Restricted)</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
-        <is>
-          <t>Sales Price (Dummy - Restricted)</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4427,45 +4400,42 @@
           <t>Net 45 Days</t>
         </is>
       </c>
-      <c r="I9" t="n">
-        <v>6000000</v>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Prasanna Hegde</t>
+        </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Prasanna Hegde</t>
+          <t>Materials Manager</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Materials Manager</t>
+          <t>+91 90000 20003</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>+91 90000 20003</t>
+          <t>accounts@vijayanagarpetrochem.example</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>accounts@vijayanagarpetrochem.example</t>
+          <t>Power &amp; Process</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Power &amp; Process</t>
+          <t>5002-02-04-01</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>5002-02-04-01</t>
+          <t>Sales Price (Dummy - Restricted)</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
-        <is>
-          <t>Sales Price (Dummy - Restricted)</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4512,45 +4482,42 @@
           <t>Net 30 Days</t>
         </is>
       </c>
-      <c r="I10" t="n">
-        <v>3000000</v>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Anoop Menon</t>
+        </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Anoop Menon</t>
+          <t>Purchase Manager</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Purchase Manager</t>
+          <t>+91 90000 20004</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>+91 90000 20004</t>
+          <t>accounts@nilacement.example</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>accounts@nilacement.example</t>
+          <t>Power &amp; Process</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Power &amp; Process</t>
+          <t>5002-02-04-01</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>5002-02-04-01</t>
+          <t>Sales Price (Dummy - Restricted)</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
-        <is>
-          <t>Sales Price (Dummy - Restricted)</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4597,45 +4564,42 @@
           <t>Net 60 Days</t>
         </is>
       </c>
-      <c r="I11" t="n">
-        <v>8000000</v>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Ramana Murthy</t>
+        </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Ramana Murthy</t>
+          <t>Project Manager</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Project Manager</t>
+          <t>+91 90000 20005</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>+91 90000 20005</t>
+          <t>accounts@telanganametro.example</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>accounts@telanganametro.example</t>
+          <t>EPC &amp; Infra</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>EPC &amp; Infra</t>
+          <t>5002-02-04-01</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>5002-02-04-01</t>
+          <t>Sales Price (Dummy - Restricted)</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
-        <is>
-          <t>Sales Price (Dummy - Restricted)</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4682,45 +4646,42 @@
           <t>Net 30 Days</t>
         </is>
       </c>
-      <c r="I12" t="n">
-        <v>2000000</v>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Vignesh K</t>
+        </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Vignesh K</t>
+          <t>Purchase Manager</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Purchase Manager</t>
+          <t>+91 90000 20006</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>+91 90000 20006</t>
+          <t>accounts@hosurauto.example</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>accounts@hosurauto.example</t>
+          <t>Manufacturing</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>5002-02-04-01</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>5002-02-04-01</t>
+          <t>Sales Price (Dummy - Restricted)</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
-        <is>
-          <t>Sales Price (Dummy - Restricted)</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -4737,7 +4698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R19"/>
+  <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4748,16 +4709,15 @@
     <col width="17" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="17" customWidth="1" min="12" max="12"/>
-    <col width="36" customWidth="1" min="13" max="13"/>
-    <col width="21" customWidth="1" min="14" max="14"/>
-    <col width="17" customWidth="1" min="15" max="15"/>
-    <col width="24" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="43" customWidth="1" min="18" max="18"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="43" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4803,50 +4763,45 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Credit limit (INR)</t>
+          <t>Contact person</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Contact person</t>
+          <t>Position</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Position</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Email</t>
+          <t>BP group</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>BP group</t>
+          <t>Control account</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Control account</t>
+          <t>Price list</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Price list</t>
+          <t>TDS code</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>TDS code</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Buys / supplies</t>
         </is>
@@ -4893,50 +4848,47 @@
           <t>Net 30 Days</t>
         </is>
       </c>
-      <c r="I2" t="n">
-        <v>2500000</v>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Mahesh Gowda</t>
+        </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Mahesh Gowda</t>
+          <t>Sales Manager</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Sales Manager</t>
+          <t>+91 90000 10101</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>+91 90000 10101</t>
+          <t>accounts@tungabhadrasteel.example</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>accounts@tungabhadrasteel.example</t>
+          <t>Steel Suppliers</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Steel Suppliers</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>Purchase Price (Dummy)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
         <is>
           <t>TMT bars, structural steel (194Q pending)</t>
         </is>
@@ -4983,50 +4935,47 @@
           <t>Net 15 Days</t>
         </is>
       </c>
-      <c r="I3" t="n">
-        <v>1000000</v>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Ravi Shankar</t>
+        </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Ravi Shankar</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>+91 90000 10102</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>+91 90000 10102</t>
+          <t>accounts@chamundicement.example</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>accounts@chamundicement.example</t>
+          <t>Building Materials</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Building Materials</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Purchase Price (Dummy)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
         <is>
           <t>Cement, river sand, M-sand, aggregate</t>
         </is>
@@ -5073,50 +5022,47 @@
           <t>Net 30 Days</t>
         </is>
       </c>
-      <c r="I4" t="n">
-        <v>1000000</v>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Anil Rao</t>
+        </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Anil Rao</t>
+          <t>Sales Executive</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Sales Executive</t>
+          <t>+91 90000 10103</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>+91 90000 10103</t>
+          <t>accounts@vidyutelectricals.example</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>accounts@vidyutelectricals.example</t>
+          <t>Elec &amp; Plumbing</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Elec &amp; Plumbing</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>Purchase Price (Dummy)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R4" t="inlineStr">
         <is>
           <t>Cables, distribution boards, flood lights</t>
         </is>
@@ -5163,50 +5109,47 @@
           <t>Net 30 Days</t>
         </is>
       </c>
-      <c r="I5" t="n">
-        <v>800000</v>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Senthil Kumar</t>
+        </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Senthil Kumar</t>
+          <t>Sales Manager</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Sales Manager</t>
+          <t>+91 90000 10104</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>+91 90000 10104</t>
+          <t>accounts@jalavahinipipes.example</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>accounts@jalavahinipipes.example</t>
+          <t>Elec &amp; Plumbing</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Elec &amp; Plumbing</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Purchase Price (Dummy)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R5" t="inlineStr">
         <is>
           <t>PVC and GI pipes</t>
         </is>
@@ -5253,50 +5196,47 @@
           <t>Net 30 Days</t>
         </is>
       </c>
-      <c r="I6" t="n">
-        <v>500000</v>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Priya Patil</t>
+        </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Priya Patil</t>
+          <t>Key Account Manager</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Key Account Manager</t>
+          <t>+91 90000 10105</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>+91 90000 10105</t>
+          <t>accounts@rakshaksafety.example</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>accounts@rakshaksafety.example</t>
+          <t>Safety &amp; Consumable</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Safety &amp; Consumable</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>Purchase Price (Dummy)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R6" t="inlineStr">
         <is>
           <t>Helmets, safety shoes, harness</t>
         </is>
@@ -5343,50 +5283,47 @@
           <t>Net 15 Days</t>
         </is>
       </c>
-      <c r="I7" t="n">
-        <v>500000</v>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Manjunath H</t>
+        </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Manjunath H</t>
+          <t>Sales Executive</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Sales Executive</t>
+          <t>+91 90000 10106</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>+91 90000 10106</t>
+          <t>accounts@agniwelding.example</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>accounts@agniwelding.example</t>
+          <t>Safety &amp; Consumable</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Safety &amp; Consumable</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Purchase Price (Dummy)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
         <is>
           <t>Welding rods, cutting &amp; grinding discs</t>
         </is>
@@ -5433,50 +5370,47 @@
           <t>Net 30 Days</t>
         </is>
       </c>
-      <c r="I8" t="n">
-        <v>700000</v>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Basavaraj Patil</t>
+        </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Basavaraj Patil</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>+91 90000 10107</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>+91 90000 10107</t>
+          <t>accounts@shaktitools.example</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>accounts@shaktitools.example</t>
+          <t>Tools &amp; Equipment</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Tools &amp; Equipment</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Purchase Price (Dummy)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
         <is>
           <t>Pumps, power tools, drills, epoxy grout</t>
         </is>
@@ -5523,50 +5457,47 @@
           <t>Net 15 Days</t>
         </is>
       </c>
-      <c r="I9" t="n">
-        <v>300000</v>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Imran Khan</t>
+        </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Imran Khan</t>
+          <t>Operations Manager</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Operations Manager</t>
+          <t>+91 90000 10108</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>+91 90000 10108</t>
+          <t>accounts@sarathiroadlines.example</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>accounts@sarathiroadlines.example</t>
+          <t>Transporters</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Transporters</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Purchase Price (Dummy)</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
-        <is>
-          <t>C2</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
         <is>
           <t>Transport (GTA) - TDS 194C 2%</t>
         </is>
@@ -5613,50 +5544,47 @@
           <t>Net 30 Days</t>
         </is>
       </c>
-      <c r="I10" t="n">
-        <v>500000</v>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Ramesh R</t>
+        </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Ramesh R</t>
+          <t>Proprietor</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Proprietor</t>
+          <t>+91 90000 10109</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>+91 90000 10109</t>
+          <t>accounts@rameshfabrication.example</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>accounts@rameshfabrication.example</t>
+          <t>Subcontractors</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Subcontractors</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>Purchase Price (Dummy)</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
-        <is>
-          <t>C1</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
         <is>
           <t>Fabrication subcontracting - TDS 194C 1%</t>
         </is>
@@ -5703,45 +5631,42 @@
           <t>Net 30 Days</t>
         </is>
       </c>
-      <c r="I11" t="n">
-        <v>2500000</v>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Ganesh Rao</t>
+        </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Ganesh Rao</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>+91 90000 20101</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>+91 90000 20101</t>
+          <t>accounts@shreeganeshsteel.example</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>accounts@shreeganeshsteel.example</t>
+          <t>Steel Suppliers</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Steel Suppliers</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
-        <is>
-          <t>Purchase Price (Dummy)</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
         <is>
           <t>Q01</t>
         </is>
@@ -5788,45 +5713,42 @@
           <t>Net 45 Days</t>
         </is>
       </c>
-      <c r="I12" t="n">
-        <v>5000000</v>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Srinivas Rao</t>
+        </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Srinivas Rao</t>
+          <t>Sales Manager</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Sales Manager</t>
+          <t>+91 90000 20102</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>+91 90000 20102</t>
+          <t>accounts@deccanstructural.example</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>accounts@deccanstructural.example</t>
+          <t>Steel Suppliers</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Steel Suppliers</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
-        <is>
-          <t>Purchase Price (Dummy)</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
         <is>
           <t>Q01</t>
         </is>
@@ -5873,45 +5795,42 @@
           <t>Net 30 Days</t>
         </is>
       </c>
-      <c r="I13" t="n">
-        <v>2000000</v>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Arun Prakash</t>
+        </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Arun Prakash</t>
+          <t>Sales Head</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Sales Head</t>
+          <t>+91 90000 20103</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>+91 90000 20103</t>
+          <t>accounts@kaverialloys.example</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>accounts@kaverialloys.example</t>
+          <t>Steel Suppliers</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Steel Suppliers</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
-        <is>
-          <t>Purchase Price (Dummy)</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -5958,45 +5877,42 @@
           <t>Net 15 Days</t>
         </is>
       </c>
-      <c r="I14" t="n">
-        <v>500000</v>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Nagaraj N</t>
+        </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Nagaraj N</t>
+          <t>Proprietor</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Proprietor</t>
+          <t>+91 90000 20104</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>+91 90000 20104</t>
+          <t>accounts@nandiwelding.example</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>accounts@nandiwelding.example</t>
+          <t>Safety &amp; Consumable</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Safety &amp; Consumable</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
-        <is>
-          <t>Purchase Price (Dummy)</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6043,45 +5959,42 @@
           <t>Net 15 Days</t>
         </is>
       </c>
-      <c r="I15" t="n">
-        <v>500000</v>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Kiran Kumar</t>
+        </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Kiran Kumar</t>
+          <t>Plant Manager</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Plant Manager</t>
+          <t>+91 90000 20105</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>+91 90000 20105</t>
+          <t>accounts@vayugases.example</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>accounts@vayugases.example</t>
+          <t>Safety &amp; Consumable</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Safety &amp; Consumable</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
-        <is>
-          <t>Purchase Price (Dummy)</t>
-        </is>
-      </c>
-      <c r="Q15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6128,45 +6041,42 @@
           <t>Net 30 Days</t>
         </is>
       </c>
-      <c r="I16" t="n">
-        <v>500000</v>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Sneha Joshi</t>
+        </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Sneha Joshi</t>
+          <t>Sales Manager</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Sales Manager</t>
+          <t>+91 90000 20106</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>+91 90000 20106</t>
+          <t>accounts@surakshasafety.example</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>accounts@surakshasafety.example</t>
+          <t>Safety &amp; Consumable</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Safety &amp; Consumable</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
-        <is>
-          <t>Purchase Price (Dummy)</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -6213,45 +6123,42 @@
           <t>Net 30 Days</t>
         </is>
       </c>
-      <c r="I17" t="n">
-        <v>500000</v>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Bharath B</t>
+        </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Bharath B</t>
+          <t>Proprietor</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Proprietor</t>
+          <t>+91 90000 20107</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>+91 90000 20107</t>
+          <t>accounts@bharathicoating.example</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>accounts@bharathicoating.example</t>
+          <t>Subcontractors</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Subcontractors</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
-        <is>
-          <t>Purchase Price (Dummy)</t>
-        </is>
-      </c>
-      <c r="Q17" t="inlineStr">
         <is>
           <t>C1</t>
         </is>
@@ -6298,45 +6205,42 @@
           <t>Net 15 Days</t>
         </is>
       </c>
-      <c r="I18" t="n">
-        <v>300000</v>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Mohammed Rafi</t>
+        </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Mohammed Rafi</t>
+          <t>Operations Manager</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Operations Manager</t>
+          <t>+91 90000 20108</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>+91 90000 20108</t>
+          <t>accounts@mysorefreight.example</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>accounts@mysorefreight.example</t>
+          <t>Transporters</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Transporters</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
-        <is>
-          <t>Purchase Price (Dummy)</t>
-        </is>
-      </c>
-      <c r="Q18" t="inlineStr">
         <is>
           <t>C2</t>
         </is>
@@ -6383,45 +6287,42 @@
           <t>Net 30 Days</t>
         </is>
       </c>
-      <c r="I19" t="n">
-        <v>200000</v>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Prakash S</t>
+        </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Prakash S</t>
+          <t>Partner</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Partner</t>
+          <t>+91 90000 20109</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>+91 90000 20109</t>
+          <t>accounts@prakashassociates.example</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>accounts@prakashassociates.example</t>
+          <t>Consultants</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Consultants</t>
+          <t>3002-02-01</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>3002-02-01</t>
+          <t>Purchase Price (Dummy)</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
-        <is>
-          <t>Purchase Price (Dummy)</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
         <is>
           <t>J10</t>
         </is>

</xml_diff>

<commit_message>
P2P and O2C training demos, quotation comparison and PO receipt reports, credit/conversion G/L fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/u1_masters/U1_Master_Data.xlsx
+++ b/data/u1_masters/U1_Master_Data.xlsx
@@ -2306,7 +2306,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -2357,6 +2357,9 @@
       </c>
       <c r="Q14" t="n">
         <v>190</v>
+      </c>
+      <c r="R14" t="n">
+        <v>250</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -3651,7 +3654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3670,7 +3673,7 @@
     <col width="17" customWidth="1" min="14" max="14"/>
     <col width="34" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="42" customWidth="1" min="17" max="17"/>
+    <col width="48" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4198,62 +4201,62 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C0001</t>
+          <t>U1C006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Sahyadri Infra Projects Pvt Ltd</t>
+          <t>ABC Developers Pvt Ltd</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Sahyadri House, 7th Floor, Bandra Kurla Complex, Bandra East, Mumbai - 400051</t>
+          <t>No. 21, ABC Towers, 4th Floor, Outer Ring Road, Marathahalli, Bengaluru - 560037</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Site - Navi Mumbai Logistics Hub: Plot 18, TTC Industrial Area, Mahape, Navi Mumbai - 400710</t>
+          <t>Site - ABC Residency Towers: Sy. No. 54, Sarjapur Road, Dommasandra, Bengaluru - 562125</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Maharashtra</t>
+          <t>Karnataka</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>27AAGCS6631P1ZQ</t>
+          <t>29AABCA7781K1Z6</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>AAGCS6631P</t>
+          <t>AABCA7781K</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Net 45 Days</t>
+          <t>Net 30 Days</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Rahul Shinde</t>
+          <t>Naveen Shetty</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Procurement Manager</t>
+          <t>Purchase Manager</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>+91 90000 20001</t>
+          <t>+91 90000 10006</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>accounts@sahyadriinfra.example</t>
+          <t>accounts@abcdevelopers.example</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -4274,73 +4277,78 @@
       <c r="P7" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Residential towers - TMT bars, safety items (O2C demo)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C0002</t>
+          <t>C0001</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Coromandel Power Engineering Ltd</t>
+          <t>Sahyadri Infra Projects Pvt Ltd</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Coromandel Towers, 4th Floor, Mount Road, Nandanam, Chennai - 600035</t>
+          <t>Sahyadri House, 7th Floor, Bandra Kurla Complex, Bandra East, Mumbai - 400051</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Site - Ennore Power Station: Ennore Port Road, Ennore, Ennore, Chennai - 600057</t>
+          <t>Site - Navi Mumbai Logistics Hub: Plot 18, TTC Industrial Area, Mahape, Navi Mumbai - 400710</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Tamil Nadu</t>
+          <t>Maharashtra</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>33AABCC8842H1ZQ</t>
+          <t>27AAGCS6631P1ZQ</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>AABCC8842H</t>
+          <t>AAGCS6631P</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Net 60 Days</t>
+          <t>Net 45 Days</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Ganesan R</t>
+          <t>Rahul Shinde</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Purchase Manager</t>
+          <t>Procurement Manager</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>+91 90000 20002</t>
+          <t>+91 90000 20001</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>accounts@coromandelpower.example</t>
+          <t>accounts@sahyadriinfra.example</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Power &amp; Process</t>
+          <t>EPC &amp; Infra</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -4362,62 +4370,62 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C0003</t>
+          <t>C0002</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Vijayanagar Petrochem Industries Ltd</t>
+          <t>Coromandel Power Engineering Ltd</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Vijayanagar Petrochem Complex, Sandur Road, Toranagallu, Ballari - 583123</t>
+          <t>Coromandel Towers, 4th Floor, Mount Road, Nandanam, Chennai - 600035</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Site - Refinery Expansion: Plant Gate 3, Sandur Road, Toranagallu, Ballari - 583123</t>
+          <t>Site - Ennore Power Station: Ennore Port Road, Ennore, Ennore, Chennai - 600057</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Karnataka</t>
+          <t>Tamil Nadu</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>29AACCV2207N1Z3</t>
+          <t>33AABCC8842H1ZQ</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>AACCV2207N</t>
+          <t>AABCC8842H</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Net 45 Days</t>
+          <t>Net 60 Days</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Prasanna Hegde</t>
+          <t>Ganesan R</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Materials Manager</t>
+          <t>Purchase Manager</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>+91 90000 20003</t>
+          <t>+91 90000 20002</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>accounts@vijayanagarpetrochem.example</t>
+          <t>accounts@coromandelpower.example</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -4444,62 +4452,62 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C0004</t>
+          <t>C0003</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Nila Cement Works Pvt Ltd</t>
+          <t>Vijayanagar Petrochem Industries Ltd</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Nila Cement Works, Kanjikode Industrial Area, Kanjikode, Palakkad - 678621</t>
+          <t>Vijayanagar Petrochem Complex, Sandur Road, Toranagallu, Ballari - 583123</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Site - Kiln Upgrade: Plant Gate 1, Kanjikode Industrial Area, Kanjikode, Palakkad - 678621</t>
+          <t>Site - Refinery Expansion: Plant Gate 3, Sandur Road, Toranagallu, Ballari - 583123</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Kerala</t>
+          <t>Karnataka</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>32AAICN4419D1ZT</t>
+          <t>29AACCV2207N1Z3</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>AAICN4419D</t>
+          <t>AACCV2207N</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Net 30 Days</t>
+          <t>Net 45 Days</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Anoop Menon</t>
+          <t>Prasanna Hegde</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Purchase Manager</t>
+          <t>Materials Manager</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>+91 90000 20004</t>
+          <t>+91 90000 20003</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>accounts@nilacement.example</t>
+          <t>accounts@vijayanagarpetrochem.example</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -4526,67 +4534,67 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C0005</t>
+          <t>C0004</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Telangana Urban Metro Contractors</t>
+          <t>Nila Cement Works Pvt Ltd</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Plot 45, Metro Bhavan, Begumpet Road, Begumpet, Hyderabad - 500016</t>
+          <t>Nila Cement Works, Kanjikode Industrial Area, Kanjikode, Palakkad - 678621</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Site - Metro Phase 2 Depot: Sy. No. 301, Miyapur Depot Road, Miyapur, Hyderabad - 500049</t>
+          <t>Site - Kiln Upgrade: Plant Gate 1, Kanjikode Industrial Area, Kanjikode, Palakkad - 678621</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Telangana</t>
+          <t>Kerala</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>36AAFFT7753G1ZV</t>
+          <t>32AAICN4419D1ZT</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>AAFFT7753G</t>
+          <t>AAICN4419D</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Net 60 Days</t>
+          <t>Net 30 Days</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Ramana Murthy</t>
+          <t>Anoop Menon</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Project Manager</t>
+          <t>Purchase Manager</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>+91 90000 20005</t>
+          <t>+91 90000 20004</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>accounts@telanganametro.example</t>
+          <t>accounts@nilacement.example</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>EPC &amp; Infra</t>
+          <t>Power &amp; Process</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -4608,80 +4616,162 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>C0005</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Telangana Urban Metro Contractors</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Plot 45, Metro Bhavan, Begumpet Road, Begumpet, Hyderabad - 500016</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Site - Metro Phase 2 Depot: Sy. No. 301, Miyapur Depot Road, Miyapur, Hyderabad - 500049</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>36AAFFT7753G1ZV</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>AAFFT7753G</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Net 60 Days</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Ramana Murthy</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Project Manager</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>+91 90000 20005</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>accounts@telanganametro.example</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>EPC &amp; Infra</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>5002-02-04-01</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Sales Price (Dummy - Restricted)</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>C0006</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Hosur Auto Components Pvt Ltd</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Plot 88, SIPCOT Phase I, Bagalur Road, SIPCOT Industrial Area, Hosur - 635126</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Plant 2: Plot 92, SIPCOT Phase II, Mookandapalli, Hosur - 635126</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Tamil Nadu</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>33AAHCH3398F1ZI</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>AAHCH3398F</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>Net 30 Days</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Vignesh K</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Purchase Manager</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>+91 90000 20006</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>accounts@hosurauto.example</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>Manufacturing</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>5002-02-04-01</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>Sales Price (Dummy - Restricted)</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
+      <c r="P13" t="inlineStr">
         <is>
           <t>-</t>
         </is>

</xml_diff>

<commit_message>
Renumber U1 BPs to C0008-C0011 / V0011-V0018 and group BPs by GST place of supply
Customers: Intrastate / Interstate / Export; vendors: Intrastate Vendor / Interstate Vendor / Import Vendor.
U1C006 -> C0012 and U1V001 -> V0010 have transactions and are renamed in the SAP client.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/u1_masters/U1_Master_Data.xlsx
+++ b/data/u1_masters/U1_Master_Data.xlsx
@@ -3657,7 +3657,7 @@
   <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
@@ -3669,7 +3669,7 @@
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
     <col width="39" customWidth="1" min="12" max="12"/>
-    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
     <col width="17" customWidth="1" min="14" max="14"/>
     <col width="34" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
@@ -3766,7 +3766,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>U1C001</t>
+          <t>C0007</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3826,7 +3826,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>EPC &amp; Infra</t>
+          <t>Intrastate</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -3853,7 +3853,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>U1C002</t>
+          <t>C0008</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Industrial Developer</t>
+          <t>Intrastate</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -3940,7 +3940,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>U1C003</t>
+          <t>C0009</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -4000,7 +4000,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Power &amp; Process</t>
+          <t>Interstate</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -4027,7 +4027,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>U1C004</t>
+          <t>C0010</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -4087,7 +4087,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Industrial Developer</t>
+          <t>Interstate</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -4114,7 +4114,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>U1C005</t>
+          <t>C0011</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -4174,7 +4174,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>EPC &amp; Infra</t>
+          <t>Interstate</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -4201,7 +4201,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>U1C006</t>
+          <t>C0012</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4261,7 +4261,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>EPC &amp; Infra</t>
+          <t>Intrastate</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -4348,7 +4348,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>EPC &amp; Infra</t>
+          <t>Interstate</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -4430,7 +4430,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Power &amp; Process</t>
+          <t>Interstate</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -4512,7 +4512,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Power &amp; Process</t>
+          <t>Intrastate</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -4594,7 +4594,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Power &amp; Process</t>
+          <t>Interstate</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -4676,7 +4676,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>EPC &amp; Infra</t>
+          <t>Interstate</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -4758,7 +4758,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Manufacturing</t>
+          <t>Interstate</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -4791,7 +4791,7 @@
   <dimension ref="A1:Q19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
@@ -4803,7 +4803,7 @@
     <col width="21" customWidth="1" min="10" max="10"/>
     <col width="17" customWidth="1" min="11" max="11"/>
     <col width="36" customWidth="1" min="12" max="12"/>
-    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="19" customWidth="1" min="13" max="13"/>
     <col width="17" customWidth="1" min="14" max="14"/>
     <col width="24" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
@@ -4900,7 +4900,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>U1V001</t>
+          <t>V0010</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -4960,7 +4960,7 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Steel Suppliers</t>
+          <t>Intrastate Vendor</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -4987,7 +4987,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>U1V002</t>
+          <t>V0011</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5047,7 +5047,7 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Building Materials</t>
+          <t>Intrastate Vendor</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -5074,7 +5074,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>U1V003</t>
+          <t>V0012</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -5134,7 +5134,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Elec &amp; Plumbing</t>
+          <t>Intrastate Vendor</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -5161,7 +5161,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>U1V004</t>
+          <t>V0013</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -5221,7 +5221,7 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Elec &amp; Plumbing</t>
+          <t>Interstate Vendor</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -5248,7 +5248,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>U1V005</t>
+          <t>V0014</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Safety &amp; Consumable</t>
+          <t>Interstate Vendor</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -5335,7 +5335,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>U1V006</t>
+          <t>V0015</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Safety &amp; Consumable</t>
+          <t>Intrastate Vendor</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -5422,7 +5422,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>U1V007</t>
+          <t>V0016</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -5482,7 +5482,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Tools &amp; Equipment</t>
+          <t>Intrastate Vendor</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -5509,7 +5509,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>U1V008</t>
+          <t>V0017</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Transporters</t>
+          <t>Intrastate Vendor</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -5596,7 +5596,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>U1V009</t>
+          <t>V0018</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -5656,7 +5656,7 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Subcontractors</t>
+          <t>Intrastate Vendor</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -5743,7 +5743,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Steel Suppliers</t>
+          <t>Intrastate Vendor</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -5825,7 +5825,7 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Steel Suppliers</t>
+          <t>Interstate Vendor</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -5907,7 +5907,7 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Steel Suppliers</t>
+          <t>Interstate Vendor</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -5989,7 +5989,7 @@
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Safety &amp; Consumable</t>
+          <t>Intrastate Vendor</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -6071,7 +6071,7 @@
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Safety &amp; Consumable</t>
+          <t>Intrastate Vendor</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -6153,7 +6153,7 @@
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Safety &amp; Consumable</t>
+          <t>Interstate Vendor</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -6235,7 +6235,7 @@
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Subcontractors</t>
+          <t>Intrastate Vendor</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -6317,7 +6317,7 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Transporters</t>
+          <t>Intrastate Vendor</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -6399,7 +6399,7 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Consultants</t>
+          <t>Intrastate Vendor</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">

</xml_diff>

<commit_message>
Consumables items on UoM group Each / NOS
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/u1_masters/U1_Master_Data.xlsx
+++ b/data/u1_masters/U1_Master_Data.xlsx
@@ -1270,7 +1270,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1390,7 +1390,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>LTR</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -3223,27 +3223,27 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>ELECTRODE</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Box</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
@@ -3319,7 +3319,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>DISC</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -3329,7 +3329,7 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Box</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -3415,7 +3415,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>DISC</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Box</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -3703,27 +3703,27 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>VOLUME</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>LTR</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>LTR</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>LTR</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>LTR</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
@@ -4747,27 +4747,27 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>AREA</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Square Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Square Feet</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Square Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Square Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
@@ -4840,27 +4840,27 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>VOLUME</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>LTR</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>LTR</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>LTR</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>LTR</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
@@ -4933,27 +4933,27 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>WEIGHT</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Grams</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Grams</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Grams</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Grams</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -5031,22 +5031,22 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Pairs</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Pairs</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Pairs</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Pairs</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
@@ -5119,27 +5119,27 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>VOLUME</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>LTR</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>LTR</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>LTR</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>LTR</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">

</xml_diff>

<commit_message>
All items without transactions on UoM group Each / NOS
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/u1_masters/U1_Master_Data.xlsx
+++ b/data/u1_masters/U1_Master_Data.xlsx
@@ -1153,7 +1153,7 @@
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
     <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1240,7 +1240,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1480,7 +1480,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Square Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Square Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1600,10 +1600,10 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="19" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
-    <col width="19" customWidth="1" min="11" max="11"/>
+    <col width="5" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
     <col width="19" customWidth="1" min="12" max="12"/>
     <col width="18" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
@@ -1855,27 +1855,27 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>WEIGHT</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -1954,27 +1954,27 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>WEIGHT</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -2053,27 +2053,27 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>CEMENT</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Bag</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Bag</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Bag</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Bag</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -2149,27 +2149,27 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>WEIGHT</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -2245,27 +2245,27 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>WEIGHT</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -2341,27 +2341,27 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>WEIGHT</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -2437,27 +2437,27 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>LENGTH</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -2734,27 +2734,27 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>LENGTH</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Feet</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
@@ -2833,27 +2833,27 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>LENGTH</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
@@ -3132,22 +3132,22 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
@@ -3612,22 +3612,22 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -3991,27 +3991,27 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>WEIGHT</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
@@ -4084,27 +4084,27 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>WEIGHT</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
@@ -4180,27 +4180,27 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>WEIGHT</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Tonnes</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
@@ -4372,27 +4372,27 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>AREA</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Square Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Square Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Square Feet</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Square Feet</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
@@ -4468,27 +4468,27 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>AREA</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Square Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Square Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Square Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Square Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
@@ -4561,27 +4561,27 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>LENGTH</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
@@ -4654,27 +4654,27 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>VOLUME</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Cubic Meters (m3)</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Cubic Meters (m3)</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Cubic Meters (m3)</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Cubic Meters (m3)</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Packet</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -5409,22 +5409,22 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Set</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Packet</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -5686,27 +5686,27 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>WEIGHT</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>KGS</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
@@ -5968,27 +5968,27 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>AREA</t>
+          <t>EACH</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Square Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Square Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Square Feet</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Square Meters</t>
+          <t>NOS</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">

</xml_diff>

<commit_message>
Add 9 Unit-1 warehouses U1 WH1-WH9
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/u1_masters/U1_Master_Data.xlsx
+++ b/data/u1_masters/U1_Master_Data.xlsx
@@ -430,11 +430,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -554,6 +554,159 @@
       <c r="C7" t="inlineStr">
         <is>
           <t>5002-01-01-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>U1 WH1</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Unit-1 Raw Material Warehouse</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>5002-01-01-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>U1 WH2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Unit-1 Bin Storage Warehouse</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>5002-01-01-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>U1 WH3</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Unit-1 Subcontractor Warehouse</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>5002-01-01-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>U1 WH4</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Unit-1 Work In Progress Warehouse</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>5002-01-01-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Unit-1 Finished Goods Warehouse</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>5002-01-01-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>U1 WH6</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Unit-1 Rework Warehouse</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>5002-01-01-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>U1 WH7</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Unit-1 Scrap Warehouse</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>5002-01-01-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>U1 WH8</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Unit-1 Cutting Warehouse</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>5002-01-01-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>U1 WH9</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Unit-1 Quality Warehouse</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>5002-01-01-06</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Retire duplicate U1 warehouses (U1WH02/03/06/07 -> U1 WH1/WH9/WH7/WH5)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/u1_masters/U1_Master_Data.xlsx
+++ b/data/u1_masters/U1_Master_Data.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -475,12 +475,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1WH04</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Raw Material Store</t>
+          <t>Rejected Warehouse</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -492,12 +492,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>U1WH03</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Quality Warehouse</t>
+          <t>Unit-1 Raw Material Warehouse</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -509,12 +509,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>U1WH04</t>
+          <t>U1 WH2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Rejected Warehouse</t>
+          <t>Unit-1 Bin Storage Warehouse</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -526,12 +526,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>U1WH06</t>
+          <t>U1 WH3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Rejected Warehouse 2 (Scrap)</t>
+          <t>Unit-1 Subcontractor Warehouse</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -543,46 +543,46 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Finished Warehouse</t>
+          <t>Unit-1 Work In Progress Warehouse</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>5002-01-01-03</t>
+          <t>5002-01-01-06</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>U1 WH1</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Unit-1 Raw Material Warehouse</t>
+          <t>Unit-1 Finished Goods Warehouse</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>5002-01-01-06</t>
+          <t>5002-01-01-03</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>U1 WH2</t>
+          <t>U1 WH6</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Unit-1 Bin Storage Warehouse</t>
+          <t>Unit-1 Rework Warehouse</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -594,12 +594,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>U1 WH3</t>
+          <t>U1 WH7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Unit-1 Subcontractor Warehouse</t>
+          <t>Unit-1 Scrap Warehouse</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -611,12 +611,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>U1 WH4</t>
+          <t>U1 WH8</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Unit-1 Work In Progress Warehouse</t>
+          <t>Unit-1 Cutting Warehouse</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -628,83 +628,15 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>U1 WH5</t>
+          <t>U1 WH9</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Unit-1 Finished Goods Warehouse</t>
+          <t>Unit-1 Quality Warehouse</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
-        <is>
-          <t>5002-01-01-03</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>U1 WH6</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Unit-1 Rework Warehouse</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>5002-01-01-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>U1 WH7</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>Unit-1 Scrap Warehouse</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>5002-01-01-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>U1 WH8</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Unit-1 Cutting Warehouse</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>5002-01-01-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>U1 WH9</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Unit-1 Quality Warehouse</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
         <is>
           <t>5002-01-01-06</t>
         </is>
@@ -1368,7 +1300,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
     </row>
@@ -1398,7 +1330,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1372,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1470,7 +1402,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1488,7 +1420,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1432,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1518,7 +1450,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
     </row>
@@ -1530,7 +1462,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1560,7 +1492,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1590,7 +1522,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1620,7 +1552,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1638,7 +1570,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
     </row>
@@ -1650,7 +1582,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1668,7 +1600,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
     </row>
@@ -1680,7 +1612,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1698,7 +1630,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1642,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1728,7 +1660,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1866,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -2033,7 +1965,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -2132,7 +2064,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -2231,7 +2163,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -2327,7 +2259,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -2423,7 +2355,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -2519,7 +2451,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -2615,7 +2547,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -2714,7 +2646,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -2813,7 +2745,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -2912,7 +2844,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -3011,7 +2943,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -3881,7 +3813,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -4262,7 +4194,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -4358,7 +4290,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -4454,7 +4386,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -4550,7 +4482,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -4646,7 +4578,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -4739,7 +4671,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -4832,7 +4764,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -5390,7 +5322,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -5486,7 +5418,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -5582,7 +5514,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>U1WH02</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -6050,7 +5982,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -6146,7 +6078,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>U1WH07</t>
+          <t>U1 WH5</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">

</xml_diff>

<commit_message>
Production BOM PL01 Anchor Bolt Plate with scrap by-product and backflushed resources
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/u1_masters/U1_Master_Data.xlsx
+++ b/data/u1_masters/U1_Master_Data.xlsx
@@ -11,10 +11,11 @@
     <sheet name="UoM" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="UoM Groups" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Item Groups" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="BOMs" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Items" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Customers" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Vendors" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Resources" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="BOMs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Items" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Customers" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Vendors" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1105,7 +1106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -1215,6 +1216,18 @@
         </is>
       </c>
       <c r="B9" t="inlineStr">
+        <is>
+          <t>RM Plates</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Scrap</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>RM Plates</t>
         </is>
@@ -1231,436 +1244,140 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="6" customWidth="1" min="4" max="4"/>
-    <col width="5" customWidth="1" min="5" max="5"/>
-    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Parent</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Cost per minute</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Warehouse</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Component</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>UoM</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Component warehouse</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SA001</t>
+          <t>RESPCM2-U1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>U1WH01</t>
+          <t>CNC Plasma With Dual Torch</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>RM003</t>
+          <t>rtMachine</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>6.5</v>
+        <v>20</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>U1 WH1</t>
+          <t>U1 WH4</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SA001</t>
+          <t>RESPCO-U1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>U1WH01</t>
+          <t>Plasma Cutting Operator</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>RM010</t>
+          <t>rtLabor</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.2</v>
+        <v>6</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>U1 WH1</t>
+          <t>U1 WH4</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SA001</t>
+          <t>RESHRO-U1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>U1WH01</t>
+          <t>Helper</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CN001</t>
+          <t>rtLabor</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.3</v>
+        <v>4</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>U1WH01</t>
+          <t>U1 WH4</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FG004</t>
+          <t>RESGGM-U1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>U1 WH5</t>
+          <t>Grinding Machine</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SA001</t>
+          <t>rtMachine</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>U1WH01</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>FG004</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>U1 WH5</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>BO001</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>U1 WH1</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>FG004</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>U1 WH5</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>BO002</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>8</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>U1 WH1</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>FG004</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>U1 WH5</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>CN005</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>U1WH01</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>FG004</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>U1 WH5</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>PM001</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>4</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>U1WH01</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>FG004</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>U1 WH5</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>PM003</t>
-        </is>
-      </c>
-      <c r="D10" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>U1WH01</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>FG005</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>U1 WH5</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>RM008</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>U1 WH1</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>FG005</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>U1 WH5</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>RM009</t>
-        </is>
-      </c>
-      <c r="D12" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>U1 WH1</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>FG005</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>U1 WH5</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>RM010</t>
-        </is>
-      </c>
-      <c r="D13" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>U1 WH1</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>FG005</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>U1 WH5</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>BO002</t>
-        </is>
-      </c>
-      <c r="D14" t="n">
-        <v>4</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>NOS</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>U1 WH1</t>
+          <t>U1 WH4</t>
         </is>
       </c>
     </row>
@@ -1675,10 +1392,942 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U46"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Parent</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Warehouse</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Seq</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>UoM</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Component warehouse</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Issue method</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SA001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>U1WH01</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>RM003</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>U1 WH1</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SA001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>U1WH01</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>RM010</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>U1 WH1</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SA001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>U1WH01</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>CN001</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>U1WH01</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>FG004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>SA001</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>U1WH01</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>FG004</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>BO001</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>U1 WH1</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FG004</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BO002</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>8</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>U1 WH1</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>FG004</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>CN005</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>U1WH01</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>FG004</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>PM001</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>U1WH01</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FG004</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>6</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>PM003</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>U1WH01</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>FG005</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>RM008</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>U1 WH1</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>FG005</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>RM009</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>U1 WH1</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>FG005</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>RM010</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>U1 WH1</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FG005</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>BO002</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>U1 WH1</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PL01</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Z24631250005</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>KGS</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>U1 WH8</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PL01</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>SCR220001</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>KGS</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>U1 WH7</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Backflush</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>PL01</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>3</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Resource</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>RESPCM2-U1</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Mins</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>U1 WH4</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Backflush</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>PL01</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Resource</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>RESPCO-U1</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Mins</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>U1 WH4</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Backflush</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>PL01</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>5</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Resource</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>RESHRO-U1</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Mins</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>U1 WH4</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Backflush</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>PL01</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>6</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Resource</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>RESGGM-U1</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Mins</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>U1 WH4</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Backflush</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>PL01</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>7</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Resource</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>RESHRO-U1</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Mins</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>U1 WH4</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Backflush</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -6023,17 +6672,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>FG005</t>
+          <t>Z24631250005</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Insulated Roof Panel Assembly</t>
+          <t>HR Plate, IS:2062 Gr. BR / S355JR, Size: 1250 x 5 mm</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Finished Goods</t>
+          <t>Raw material</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -6043,52 +6692,52 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>EACH</t>
+          <t>WEIGHT</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>NOS</t>
+          <t>KGS</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>NOS</t>
+          <t>KGS</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>NOS</t>
+          <t>KGS</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>NOS</t>
+          <t>KGS</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>U1 WH5</t>
+          <t>U1 WH1</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>Standard</t>
+          <t>Moving Average</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>7308</t>
+          <t>7208</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
@@ -6099,18 +6748,300 @@
       <c r="P46" t="n">
         <v>18</v>
       </c>
-      <c r="Q46" t="n">
+      <c r="R46" t="n">
+        <v>62</v>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>SCR220001</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>MS Scrap melting</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Scrap</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>WEIGHT</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>KGS</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>KGS</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>KGS</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>KGS</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>U1 WH7</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>Moving Average</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>7204</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Regular (Goods)</t>
+        </is>
+      </c>
+      <c r="P47" t="n">
+        <v>18</v>
+      </c>
+      <c r="S47" t="n">
+        <v>32</v>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>PL01</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Anchor Bolt Plate</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Finished Goods</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>EACH</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>7308</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Regular (Goods)</t>
+        </is>
+      </c>
+      <c r="P48" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>43</v>
+      </c>
+      <c r="S48" t="n">
+        <v>60</v>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>FG005</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Insulated Roof Panel Assembly</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Finished Goods</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>EACH</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>NOS</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>U1 WH5</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>7308</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Regular (Goods)</t>
+        </is>
+      </c>
+      <c r="P49" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q49" t="n">
         <v>1250</v>
       </c>
-      <c r="S46" t="n">
+      <c r="S49" t="n">
         <v>1650</v>
       </c>
-      <c r="T46" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="U46" t="inlineStr">
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
         <is>
           <t>N</t>
         </is>
@@ -6121,7 +7052,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7255,7 +8186,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>